<commit_message>
Atualiza relatorios e adiciona novas rotinas
</commit_message>
<xml_diff>
--- a/data/dRevendas.xlsx
+++ b/data/dRevendas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cadcom.patos\Documents\promax-web-driver\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36D8BE85-6316-45B8-BA9D-54264860EE4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41DBAF80-AC1F-485B-A830-7D59351E8B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="34">
   <si>
     <t>SOUSA</t>
   </si>
@@ -136,6 +136,9 @@
   </si>
   <si>
     <t>nomeUnidade020502</t>
+  </si>
+  <si>
+    <t>SUMÉ</t>
   </si>
 </sst>
 </file>
@@ -654,7 +657,7 @@
         <v>3</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="L5" s="1" t="s">
         <v>14</v>

</xml_diff>